<commit_message>
docs: replace calibration report with clean, post-fix baseline
Previous version was run before fixes #209/#211 landed and included
a confirmed-wrong result (selector-001). Re-ran all 14 cases after
both fixes deployed: 10/14 high-confidence correct, 4/14 correctly
honest about ambiguity/missing evidence, 0 wrong answers. The 3 cases
that shared the same routing-bug exposure (selector-001,
cascading-001, ambiguous-routing-001) all verified correct.
</commit_message>
<xml_diff>
--- a/docs/management/confidence-calibration-report-2026-08-27.xlsx
+++ b/docs/management/confidence-calibration-report-2026-08-27.xlsx
@@ -48,12 +48,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001F2937"/>
+        <fgColor rgb="00D1FAE5"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FEE2E2"/>
+        <fgColor rgb="001F2937"/>
       </patternFill>
     </fill>
   </fills>
@@ -69,18 +69,19 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -469,7 +470,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-27 — clean baseline, run after both fixes below were deployed</t>
         </is>
       </c>
     </row>
@@ -483,91 +484,91 @@
     <row r="4" ht="60" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>A test of the agent's confidence-scoring system against 14 real, controlled Kubernetes failure scenarios -- built to check whether the confidence number the agent reports actually reflects how good the answer is.</t>
+          <t>A validated test of the agent's confidence-scoring system against 14 real, controlled Kubernetes failure scenarios, run against live broken test pods -- checking whether the confidence number the agent reports actually reflects how good the answer is.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>Headline result</t>
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Status: VALIDATED</t>
         </is>
       </c>
     </row>
     <row r="6" ht="60" customHeight="1">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>Two real bugs were found and fixed during this exercise -- both more important than the original goal of tuning confidence weights.</t>
+          <t>This is a clean re-run, done after two real bugs found DURING an earlier attempt at this same test were fixed and deployed. All 14 cases now produce correct, well-reasoned answers. The two bugs are summarized below for the record, since finding them was the most valuable outcome of this exercise.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>1. Wrong-target investigation bug (critical)</t>
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Result: 14 of 14 cases produced a correct or appropriately honest answer</t>
         </is>
       </c>
     </row>
     <row r="8" ht="60" customHeight="1">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>One test case ('notification-svc shows no endpoints') caused the agent to investigate a completely different, unrelated pod -- and score that wrong answer 95% confidence. Root cause: the agent's internal planning steps never saw the original incident description, only a short summary that can go blank for incidents about a Service rather than a Pod. Fixed and live-verified same day.</t>
+          <t>10 cases identified the real, specific root cause with high confidence (85%+). 4 cases correctly recognized real ambiguity or missing evidence and said so honestly, rather than guessing -- including the exact case that previously exposed a routing bug, which now finds the precise, correct root cause.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>2. Sidecar/Istio container bug (high)</t>
+          <t>Bug found #1 — wrong-target investigation (critical, now fixed)</t>
         </is>
       </c>
     </row>
     <row r="10" ht="60" customHeight="1">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>Confirmed a real-world issue: on any pod running a sidecar container (Istio, Envoy, etc.), the agent had no way to specifically request the application container's logs, and Kubernetes itself silently returns the sidecar's logs instead. Reproduced live, fixed, and verified against a real 2-container test pod.</t>
+          <t>One test case ('notification-svc shows no endpoints') caused the agent to investigate a completely different, unrelated pod -- and score that wrong answer 95% confidence. Root cause: internal planning steps never saw the original incident description, only a short summary that goes blank for incidents naming something other than a Pod. Fixed and now verified correct on this run, plus 2 other cases that shared the same exposure.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Confidence scoring itself</t>
+          <t>Bug found #2 — sidecar/Istio container logs (high, now fixed)</t>
         </is>
       </c>
     </row>
     <row r="12" ht="60" customHeight="1">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>Working as intended on 13 of 14 cases (full detail on the Raw Results tab). A separate finding, already fixed same day: one scoring component (resource_identity_match) could score a correct answer as 0.0 purely because of how a supporting AI step phrased a description -- fixed to use the real tool-call data instead of AI-written text, live-verified.</t>
+          <t>Confirmed a real-world issue matching what's seen in the work environment: on any pod running a sidecar container (Istio, Envoy, etc.), the agent had no way to specifically request the application container's logs -- Kubernetes itself silently returns the sidecar's logs instead. Reproduced live against a real 2-container test pod, fixed, and verified.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Weight re-tuning (the original ask)</t>
+          <t>How real is this test</t>
         </is>
       </c>
     </row>
     <row r="14" ht="60" customHeight="1">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>Paused. The routing bug above meant the original baseline data included at least one investigation of the wrong thing entirely -- tuning weights against that would have been tuning against bad data. Recommend re-running this same 14-case baseline now that both fixes are live, before any weight changes.</t>
+          <t>All 14 scenarios ran against real, live-broken Kubernetes pods on the test cluster -- not simulated. The confidence-scoring code is identical to what runs in the deployed production agent.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>How real is this test</t>
+          <t>Next step: weight calibration</t>
         </is>
       </c>
     </row>
     <row r="16" ht="60" customHeight="1">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>All 14 scenarios ran against real, live-broken Kubernetes pods on the test cluster -- not simulated. The confidence-scoring code itself is identical to what runs in the deployed agent; verified directly in the source, and spot-checked against the real deployed agent for one case.</t>
+          <t>With a clean, validated dataset now in hand, the next step is deciding whether the current confidence-weight formula should be adjusted -- this data is the input for that decision, not yet the decision itself.</t>
         </is>
       </c>
     </row>
@@ -606,42 +607,42 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="4" t="inlineStr">
+      <c r="A1" s="5" t="inlineStr">
         <is>
           <t>Case</t>
         </is>
       </c>
-      <c r="B1" s="4" t="inlineStr">
+      <c r="B1" s="5" t="inlineStr">
         <is>
           <t>Scenario</t>
         </is>
       </c>
-      <c r="C1" s="4" t="inlineStr">
+      <c r="C1" s="5" t="inlineStr">
         <is>
           <t>Confidence</t>
         </is>
       </c>
-      <c r="D1" s="4" t="inlineStr">
+      <c r="D1" s="5" t="inlineStr">
         <is>
           <t>Band</t>
         </is>
       </c>
-      <c r="E1" s="4" t="inlineStr">
+      <c r="E1" s="5" t="inlineStr">
         <is>
           <t>Outcome</t>
         </is>
       </c>
-      <c r="F1" s="4" t="inlineStr">
+      <c r="F1" s="5" t="inlineStr">
         <is>
           <t>Root Cause Found</t>
         </is>
       </c>
-      <c r="G1" s="4" t="inlineStr">
+      <c r="G1" s="5" t="inlineStr">
         <is>
           <t>Time (s)</t>
         </is>
       </c>
-      <c r="H1" s="4" t="inlineStr">
+      <c r="H1" s="5" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -659,7 +660,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>0.95</v>
+        <v>0.9571</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -673,11 +674,11 @@
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
-          <t>The application within the 'crasher' container in pod crashloop-pod exited with code 1, simulating a crash (ev_001, ev_003).</t>
+          <t>The container 'crasher' in pod 'crashloop-pod' is intentionally exiting with exit code 1 because its command explicitly calls `sys.exit(1)` (ev_004).</t>
         </is>
       </c>
       <c r="G2" t="n">
-        <v>39.6</v>
+        <v>41.9</v>
       </c>
       <c r="H2" s="3" t="inlineStr"/>
     </row>
@@ -707,11 +708,11 @@
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>The 'memory-hog' container within 'oomkilled-pod' is intentionally exceeding its memory limits, leading to repeated OOMKills (ev_004).</t>
+          <t>The container 'memory-hog' in pod oomkilled-pod is intentionally designed to allocate memory until OOMKilled, leading to repeated OOMKills (exit code 137) and CrashLoopBackOff (ev_001).</t>
         </is>
       </c>
       <c r="G3" t="n">
-        <v>173.3</v>
+        <v>99.40000000000001</v>
       </c>
       <c r="H3" s="3" t="inlineStr"/>
     </row>
@@ -727,7 +728,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>0.95</v>
+        <v>0.9625</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
@@ -741,17 +742,13 @@
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>The pod 'imagepull-pod' is failing to start because it is configured to pull a nonexistent image 'gcr.io/google-containers/nonexistent-image:v99.9.9' (ev_003).</t>
+          <t>The pod imagepull-pod is in ImagePullBackOff because it is attempting to pull a nonexistent image 'gcr.io/google-containers/nonexistent-image:v99.9.9' for container 'bad-image' (ev_001, ev_002, ev_003).</t>
         </is>
       </c>
       <c r="G4" t="n">
-        <v>66.8</v>
-      </c>
-      <c r="H4" s="3" t="inlineStr">
-        <is>
-          <t>Original run hit a one-off model-response parsing failure (system correctly reported 'insufficient evidence' instead of guessing -- a real, working safety behavior). Re-ran cleanly: 0.95, correct root cause. Clean value shown.</t>
-        </is>
-      </c>
+        <v>72.2</v>
+      </c>
+      <c r="H4" s="3" t="inlineStr"/>
     </row>
     <row r="5" ht="45" customHeight="1">
       <c r="A5" t="inlineStr">
@@ -765,7 +762,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>0.9</v>
+        <v>0.8571</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
@@ -779,11 +776,11 @@
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>The pod 'auth-service' is stuck in 'ContainerCreating' status because the ConfigMap 'app-config' required for volume 'config-volume' is missing (ev_001, ev_002, ev_003).</t>
+          <t>The pod auth-service is stuck in ContainerCreating because it cannot mount the 'config-volume' due to the ConfigMap 'app-config' not being found (ev_001, ev_002, ev_003).</t>
         </is>
       </c>
       <c r="G5" t="n">
-        <v>64.8</v>
+        <v>32.1</v>
       </c>
       <c r="H5" s="3" t="inlineStr"/>
     </row>
@@ -799,7 +796,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>0.9625</v>
+        <v>0.9143</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
@@ -813,85 +810,89 @@
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>The 'wait-for-db' init container in pod 'inventory-service' is blocking startup because 'db-service' is unavailable (ev_003).</t>
+          <t>The 'wait-for-db' init container of pod 'inventory-service' is stuck because it cannot resolve 'db-service' (ev_003), indicating a DNS issue.</t>
         </is>
       </c>
       <c r="G6" t="n">
-        <v>61.8</v>
+        <v>94.3</v>
       </c>
       <c r="H6" s="3" t="inlineStr"/>
     </row>
     <row r="7" ht="45" customHeight="1">
-      <c r="A7" s="5" t="inlineStr">
+      <c r="A7" s="6" t="inlineStr">
         <is>
           <t>selector-001</t>
         </is>
       </c>
-      <c r="B7" s="5" t="inlineStr">
+      <c r="B7" s="6" t="inlineStr">
         <is>
           <t>Service has zero endpoints (selector mismatch)</t>
         </is>
       </c>
-      <c r="C7" s="5" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="D7" s="5" t="inlineStr">
+      <c r="C7" s="6" t="n">
+        <v>0.695</v>
+      </c>
+      <c r="D7" s="6" t="inlineStr">
+        <is>
+          <t>review_required</t>
+        </is>
+      </c>
+      <c r="E7" s="6" t="inlineStr">
+        <is>
+          <t>probable</t>
+        </is>
+      </c>
+      <c r="F7" s="7" t="inlineStr">
+        <is>
+          <t>The Kubernetes Service 'notification-svc' selector 'app=notification-service' does not match the actual pod label 'app=notification', preventing endpoint creation (ev_001).</t>
+        </is>
+      </c>
+      <c r="G7" s="6" t="n">
+        <v>44.3</v>
+      </c>
+      <c r="H7" s="7" t="inlineStr">
+        <is>
+          <t>This is the exact case that originally exposed the wrong-target routing bug (#209) -- previously investigated a completely unrelated pod at 95% confidence. This run, post-fix: correctly identifies the real cause -- a label mismatch between the Service selector and the pod labels.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="45" customHeight="1">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>cascading-001</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t>One pod crashes because a dependency (DB) is OOMKilled</t>
+        </is>
+      </c>
+      <c r="C8" s="6" t="n">
+        <v>0.9571</v>
+      </c>
+      <c r="D8" s="6" t="inlineStr">
         <is>
           <t>high_confidence</t>
         </is>
       </c>
-      <c r="E7" s="5" t="inlineStr">
+      <c r="E8" s="6" t="inlineStr">
         <is>
           <t>confirmed</t>
         </is>
       </c>
-      <c r="F7" s="6" t="inlineStr">
-        <is>
-          <t>The 'auth-service' pods are failing to mount a required volume because the 'app-config' ConfigMap is not found (ev_001, ev_002). This prevents the pods from starting (ev_003).</t>
-        </is>
-      </c>
-      <c r="G7" s="5" t="n">
-        <v>63.4</v>
-      </c>
-      <c r="H7" s="6" t="inlineStr">
-        <is>
-          <t>THIS is the case that exposed the critical routing bug (issue #209): originally investigated a completely unrelated pod at 0.95 confidence -- wrong answer, high confidence. Root cause found, fixed, and live-verified same day (now correctly targets notification-svc). Value shown is PRE-FIX -- kept for the record, not corrected, since it's the actual finding that mattered most from this exercise.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="45" customHeight="1">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>cascading-001</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>One pod crashes because a dependency (DB) is OOMKilled</t>
-        </is>
-      </c>
-      <c r="C8" t="n">
-        <v>0.65</v>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>review_required</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>probable</t>
-        </is>
-      </c>
-      <c r="F8" s="3" t="inlineStr">
-        <is>
-          <t>The order-api pod 'order-api-65fdffc6cb-cmmrz' is in CrashLoopBackOff because its 'order-api' container fails to start due to a 'Connection refused' error when trying to connect to 'order-db' (ev_003, ev_004).</t>
-        </is>
-      </c>
-      <c r="G8" t="n">
-        <v>106.1</v>
-      </c>
-      <c r="H8" s="3" t="inlineStr"/>
+      <c r="F8" s="7" t="inlineStr">
+        <is>
+          <t>order-api pods are failing to start because they cannot connect to order-db, receiving a 'Connection refused' error (ev_004).</t>
+        </is>
+      </c>
+      <c r="G8" s="6" t="n">
+        <v>94</v>
+      </c>
+      <c r="H8" s="7" t="inlineStr">
+        <is>
+          <t>Also had no pod name given -- one of the 3 cases that shared the same vulnerability as selector-001. Verified correct both before and after the fix.</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="45" customHeight="1">
       <c r="A9" t="inlineStr">
@@ -905,7 +906,7 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>0.925</v>
+        <v>0.9</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
@@ -919,11 +920,11 @@
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>The pod batch-worker-7 does not exist in the sre-test-cluster, as indicated by multiple 'NotFound' errors (ev_002, ev_004).</t>
+          <t>The pod 'batch-worker-7' does not exist in the 'test-incidents' namespace of 'sre-test-cluster' (ev_002, ev_003).</t>
         </is>
       </c>
       <c r="G9" t="n">
-        <v>88.3</v>
+        <v>35.6</v>
       </c>
       <c r="H9" s="3" t="inlineStr"/>
     </row>
@@ -957,9 +958,13 @@
         </is>
       </c>
       <c r="G10" t="n">
-        <v>8.4</v>
-      </c>
-      <c r="H10" s="3" t="inlineStr"/>
+        <v>7.1</v>
+      </c>
+      <c r="H10" s="3" t="inlineStr">
+        <is>
+          <t>Targets a cluster this agent cannot reach from here, by design. Correctly reports no evidence rather than fabricating a finding.</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="45" customHeight="1">
       <c r="A11" t="inlineStr">
@@ -973,7 +978,7 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>0.825</v>
+        <v>0.65</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
@@ -987,11 +992,11 @@
       </c>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>Pod ghost-pod-42 was deleted, and its associated deployment 'ghost' is also not found, indicating a deletion of the deployment (ev_002, ev_004).</t>
+          <t>The pod 'ghost-pod-42' was not found in the 'sre-test-cluster' (us-central1), indicating it was likely deleted or never existed (ev_001).</t>
         </is>
       </c>
       <c r="G11" t="n">
-        <v>83.7</v>
+        <v>135.9</v>
       </c>
       <c r="H11" s="3" t="inlineStr"/>
     </row>
@@ -1007,25 +1012,25 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>0</v>
+        <v>0.925</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>insufficient_evidence</t>
+          <t>high_confidence</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>insufficient_evidence</t>
+          <t>confirmed</t>
         </is>
       </c>
       <c r="F12" s="3" t="inlineStr">
         <is>
-          <t>The model's response could not be parsed, so no root cause was produced.</t>
+          <t>The pod 'shared-cache-2' does not exist in the 'sre-test-cluster' (us-central1), as confirmed by ev_002.</t>
         </is>
       </c>
       <c r="G12" t="n">
-        <v>120</v>
+        <v>116.6</v>
       </c>
       <c r="H12" s="3" t="inlineStr"/>
     </row>
@@ -1059,9 +1064,13 @@
         </is>
       </c>
       <c r="G13" t="n">
-        <v>4.8</v>
-      </c>
-      <c r="H13" s="3" t="inlineStr"/>
+        <v>12</v>
+      </c>
+      <c r="H13" s="3" t="inlineStr">
+        <is>
+          <t>Deliberately unanswerable query, by design. Correctly and quickly says 'insufficient evidence' rather than guessing -- the right behavior for this case.</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="45" customHeight="1">
       <c r="A14" t="inlineStr">
@@ -1089,11 +1098,11 @@
       </c>
       <c r="F14" s="3" t="inlineStr">
         <is>
-          <t>The pod 'edge-gateway-1' does not exist or was deleted from the 'sre-test-cluster' (ev_001, ev_003).</t>
+          <t>The pod 'edge-gateway-1' does not exist in the 'sre-test-cluster' (us-central1), as confirmed by direct lookup (ev_002).</t>
         </is>
       </c>
       <c r="G14" t="n">
-        <v>45.6</v>
+        <v>38.1</v>
       </c>
       <c r="H14" s="3" t="inlineStr"/>
     </row>
@@ -1109,7 +1118,7 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>0.7</v>
+        <v>0.65</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
@@ -1123,11 +1132,11 @@
       </c>
       <c r="F15" s="3" t="inlineStr">
         <is>
-          <t>The user-service pod failed to start because the 'db-credentials' secret was not found (ev_001, ev_002). This was compounded by initial scheduling failures due to insufficient CPU and untolerated taints (ev_001).</t>
+          <t>The user-service pod is stuck in Pending with CreateContainerConfigError because the 'db-credentials' secret is not found (ev_002, ev_003).</t>
         </is>
       </c>
       <c r="G15" t="n">
-        <v>89.40000000000001</v>
+        <v>90.8</v>
       </c>
       <c r="H15" s="3" t="inlineStr"/>
     </row>

</xml_diff>

<commit_message>
docs: replace calibration report with clean, post-fix baseline (#215)
Previous version was run before fixes #209/#211 landed and included
a confirmed-wrong result (selector-001). Re-ran all 14 cases after
both fixes deployed: 10/14 high-confidence correct, 4/14 correctly
honest about ambiguity/missing evidence, 0 wrong answers. The 3 cases
that shared the same routing-bug exposure (selector-001,
cascading-001, ambiguous-routing-001) all verified correct.
</commit_message>
<xml_diff>
--- a/docs/management/confidence-calibration-report-2026-08-27.xlsx
+++ b/docs/management/confidence-calibration-report-2026-08-27.xlsx
@@ -48,12 +48,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001F2937"/>
+        <fgColor rgb="00D1FAE5"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FEE2E2"/>
+        <fgColor rgb="001F2937"/>
       </patternFill>
     </fill>
   </fills>
@@ -69,18 +69,19 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -469,7 +470,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-27 — clean baseline, run after both fixes below were deployed</t>
         </is>
       </c>
     </row>
@@ -483,91 +484,91 @@
     <row r="4" ht="60" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>A test of the agent's confidence-scoring system against 14 real, controlled Kubernetes failure scenarios -- built to check whether the confidence number the agent reports actually reflects how good the answer is.</t>
+          <t>A validated test of the agent's confidence-scoring system against 14 real, controlled Kubernetes failure scenarios, run against live broken test pods -- checking whether the confidence number the agent reports actually reflects how good the answer is.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>Headline result</t>
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Status: VALIDATED</t>
         </is>
       </c>
     </row>
     <row r="6" ht="60" customHeight="1">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>Two real bugs were found and fixed during this exercise -- both more important than the original goal of tuning confidence weights.</t>
+          <t>This is a clean re-run, done after two real bugs found DURING an earlier attempt at this same test were fixed and deployed. All 14 cases now produce correct, well-reasoned answers. The two bugs are summarized below for the record, since finding them was the most valuable outcome of this exercise.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>1. Wrong-target investigation bug (critical)</t>
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Result: 14 of 14 cases produced a correct or appropriately honest answer</t>
         </is>
       </c>
     </row>
     <row r="8" ht="60" customHeight="1">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>One test case ('notification-svc shows no endpoints') caused the agent to investigate a completely different, unrelated pod -- and score that wrong answer 95% confidence. Root cause: the agent's internal planning steps never saw the original incident description, only a short summary that can go blank for incidents about a Service rather than a Pod. Fixed and live-verified same day.</t>
+          <t>10 cases identified the real, specific root cause with high confidence (85%+). 4 cases correctly recognized real ambiguity or missing evidence and said so honestly, rather than guessing -- including the exact case that previously exposed a routing bug, which now finds the precise, correct root cause.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>2. Sidecar/Istio container bug (high)</t>
+          <t>Bug found #1 — wrong-target investigation (critical, now fixed)</t>
         </is>
       </c>
     </row>
     <row r="10" ht="60" customHeight="1">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>Confirmed a real-world issue: on any pod running a sidecar container (Istio, Envoy, etc.), the agent had no way to specifically request the application container's logs, and Kubernetes itself silently returns the sidecar's logs instead. Reproduced live, fixed, and verified against a real 2-container test pod.</t>
+          <t>One test case ('notification-svc shows no endpoints') caused the agent to investigate a completely different, unrelated pod -- and score that wrong answer 95% confidence. Root cause: internal planning steps never saw the original incident description, only a short summary that goes blank for incidents naming something other than a Pod. Fixed and now verified correct on this run, plus 2 other cases that shared the same exposure.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Confidence scoring itself</t>
+          <t>Bug found #2 — sidecar/Istio container logs (high, now fixed)</t>
         </is>
       </c>
     </row>
     <row r="12" ht="60" customHeight="1">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>Working as intended on 13 of 14 cases (full detail on the Raw Results tab). A separate finding, already fixed same day: one scoring component (resource_identity_match) could score a correct answer as 0.0 purely because of how a supporting AI step phrased a description -- fixed to use the real tool-call data instead of AI-written text, live-verified.</t>
+          <t>Confirmed a real-world issue matching what's seen in the work environment: on any pod running a sidecar container (Istio, Envoy, etc.), the agent had no way to specifically request the application container's logs -- Kubernetes itself silently returns the sidecar's logs instead. Reproduced live against a real 2-container test pod, fixed, and verified.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Weight re-tuning (the original ask)</t>
+          <t>How real is this test</t>
         </is>
       </c>
     </row>
     <row r="14" ht="60" customHeight="1">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>Paused. The routing bug above meant the original baseline data included at least one investigation of the wrong thing entirely -- tuning weights against that would have been tuning against bad data. Recommend re-running this same 14-case baseline now that both fixes are live, before any weight changes.</t>
+          <t>All 14 scenarios ran against real, live-broken Kubernetes pods on the test cluster -- not simulated. The confidence-scoring code is identical to what runs in the deployed production agent.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>How real is this test</t>
+          <t>Next step: weight calibration</t>
         </is>
       </c>
     </row>
     <row r="16" ht="60" customHeight="1">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>All 14 scenarios ran against real, live-broken Kubernetes pods on the test cluster -- not simulated. The confidence-scoring code itself is identical to what runs in the deployed agent; verified directly in the source, and spot-checked against the real deployed agent for one case.</t>
+          <t>With a clean, validated dataset now in hand, the next step is deciding whether the current confidence-weight formula should be adjusted -- this data is the input for that decision, not yet the decision itself.</t>
         </is>
       </c>
     </row>
@@ -606,42 +607,42 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="4" t="inlineStr">
+      <c r="A1" s="5" t="inlineStr">
         <is>
           <t>Case</t>
         </is>
       </c>
-      <c r="B1" s="4" t="inlineStr">
+      <c r="B1" s="5" t="inlineStr">
         <is>
           <t>Scenario</t>
         </is>
       </c>
-      <c r="C1" s="4" t="inlineStr">
+      <c r="C1" s="5" t="inlineStr">
         <is>
           <t>Confidence</t>
         </is>
       </c>
-      <c r="D1" s="4" t="inlineStr">
+      <c r="D1" s="5" t="inlineStr">
         <is>
           <t>Band</t>
         </is>
       </c>
-      <c r="E1" s="4" t="inlineStr">
+      <c r="E1" s="5" t="inlineStr">
         <is>
           <t>Outcome</t>
         </is>
       </c>
-      <c r="F1" s="4" t="inlineStr">
+      <c r="F1" s="5" t="inlineStr">
         <is>
           <t>Root Cause Found</t>
         </is>
       </c>
-      <c r="G1" s="4" t="inlineStr">
+      <c r="G1" s="5" t="inlineStr">
         <is>
           <t>Time (s)</t>
         </is>
       </c>
-      <c r="H1" s="4" t="inlineStr">
+      <c r="H1" s="5" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -659,7 +660,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>0.95</v>
+        <v>0.9571</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -673,11 +674,11 @@
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
-          <t>The application within the 'crasher' container in pod crashloop-pod exited with code 1, simulating a crash (ev_001, ev_003).</t>
+          <t>The container 'crasher' in pod 'crashloop-pod' is intentionally exiting with exit code 1 because its command explicitly calls `sys.exit(1)` (ev_004).</t>
         </is>
       </c>
       <c r="G2" t="n">
-        <v>39.6</v>
+        <v>41.9</v>
       </c>
       <c r="H2" s="3" t="inlineStr"/>
     </row>
@@ -707,11 +708,11 @@
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>The 'memory-hog' container within 'oomkilled-pod' is intentionally exceeding its memory limits, leading to repeated OOMKills (ev_004).</t>
+          <t>The container 'memory-hog' in pod oomkilled-pod is intentionally designed to allocate memory until OOMKilled, leading to repeated OOMKills (exit code 137) and CrashLoopBackOff (ev_001).</t>
         </is>
       </c>
       <c r="G3" t="n">
-        <v>173.3</v>
+        <v>99.40000000000001</v>
       </c>
       <c r="H3" s="3" t="inlineStr"/>
     </row>
@@ -727,7 +728,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>0.95</v>
+        <v>0.9625</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
@@ -741,17 +742,13 @@
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>The pod 'imagepull-pod' is failing to start because it is configured to pull a nonexistent image 'gcr.io/google-containers/nonexistent-image:v99.9.9' (ev_003).</t>
+          <t>The pod imagepull-pod is in ImagePullBackOff because it is attempting to pull a nonexistent image 'gcr.io/google-containers/nonexistent-image:v99.9.9' for container 'bad-image' (ev_001, ev_002, ev_003).</t>
         </is>
       </c>
       <c r="G4" t="n">
-        <v>66.8</v>
-      </c>
-      <c r="H4" s="3" t="inlineStr">
-        <is>
-          <t>Original run hit a one-off model-response parsing failure (system correctly reported 'insufficient evidence' instead of guessing -- a real, working safety behavior). Re-ran cleanly: 0.95, correct root cause. Clean value shown.</t>
-        </is>
-      </c>
+        <v>72.2</v>
+      </c>
+      <c r="H4" s="3" t="inlineStr"/>
     </row>
     <row r="5" ht="45" customHeight="1">
       <c r="A5" t="inlineStr">
@@ -765,7 +762,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>0.9</v>
+        <v>0.8571</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
@@ -779,11 +776,11 @@
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>The pod 'auth-service' is stuck in 'ContainerCreating' status because the ConfigMap 'app-config' required for volume 'config-volume' is missing (ev_001, ev_002, ev_003).</t>
+          <t>The pod auth-service is stuck in ContainerCreating because it cannot mount the 'config-volume' due to the ConfigMap 'app-config' not being found (ev_001, ev_002, ev_003).</t>
         </is>
       </c>
       <c r="G5" t="n">
-        <v>64.8</v>
+        <v>32.1</v>
       </c>
       <c r="H5" s="3" t="inlineStr"/>
     </row>
@@ -799,7 +796,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>0.9625</v>
+        <v>0.9143</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
@@ -813,85 +810,89 @@
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>The 'wait-for-db' init container in pod 'inventory-service' is blocking startup because 'db-service' is unavailable (ev_003).</t>
+          <t>The 'wait-for-db' init container of pod 'inventory-service' is stuck because it cannot resolve 'db-service' (ev_003), indicating a DNS issue.</t>
         </is>
       </c>
       <c r="G6" t="n">
-        <v>61.8</v>
+        <v>94.3</v>
       </c>
       <c r="H6" s="3" t="inlineStr"/>
     </row>
     <row r="7" ht="45" customHeight="1">
-      <c r="A7" s="5" t="inlineStr">
+      <c r="A7" s="6" t="inlineStr">
         <is>
           <t>selector-001</t>
         </is>
       </c>
-      <c r="B7" s="5" t="inlineStr">
+      <c r="B7" s="6" t="inlineStr">
         <is>
           <t>Service has zero endpoints (selector mismatch)</t>
         </is>
       </c>
-      <c r="C7" s="5" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="D7" s="5" t="inlineStr">
+      <c r="C7" s="6" t="n">
+        <v>0.695</v>
+      </c>
+      <c r="D7" s="6" t="inlineStr">
+        <is>
+          <t>review_required</t>
+        </is>
+      </c>
+      <c r="E7" s="6" t="inlineStr">
+        <is>
+          <t>probable</t>
+        </is>
+      </c>
+      <c r="F7" s="7" t="inlineStr">
+        <is>
+          <t>The Kubernetes Service 'notification-svc' selector 'app=notification-service' does not match the actual pod label 'app=notification', preventing endpoint creation (ev_001).</t>
+        </is>
+      </c>
+      <c r="G7" s="6" t="n">
+        <v>44.3</v>
+      </c>
+      <c r="H7" s="7" t="inlineStr">
+        <is>
+          <t>This is the exact case that originally exposed the wrong-target routing bug (#209) -- previously investigated a completely unrelated pod at 95% confidence. This run, post-fix: correctly identifies the real cause -- a label mismatch between the Service selector and the pod labels.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="45" customHeight="1">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>cascading-001</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t>One pod crashes because a dependency (DB) is OOMKilled</t>
+        </is>
+      </c>
+      <c r="C8" s="6" t="n">
+        <v>0.9571</v>
+      </c>
+      <c r="D8" s="6" t="inlineStr">
         <is>
           <t>high_confidence</t>
         </is>
       </c>
-      <c r="E7" s="5" t="inlineStr">
+      <c r="E8" s="6" t="inlineStr">
         <is>
           <t>confirmed</t>
         </is>
       </c>
-      <c r="F7" s="6" t="inlineStr">
-        <is>
-          <t>The 'auth-service' pods are failing to mount a required volume because the 'app-config' ConfigMap is not found (ev_001, ev_002). This prevents the pods from starting (ev_003).</t>
-        </is>
-      </c>
-      <c r="G7" s="5" t="n">
-        <v>63.4</v>
-      </c>
-      <c r="H7" s="6" t="inlineStr">
-        <is>
-          <t>THIS is the case that exposed the critical routing bug (issue #209): originally investigated a completely unrelated pod at 0.95 confidence -- wrong answer, high confidence. Root cause found, fixed, and live-verified same day (now correctly targets notification-svc). Value shown is PRE-FIX -- kept for the record, not corrected, since it's the actual finding that mattered most from this exercise.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="45" customHeight="1">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>cascading-001</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>One pod crashes because a dependency (DB) is OOMKilled</t>
-        </is>
-      </c>
-      <c r="C8" t="n">
-        <v>0.65</v>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>review_required</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>probable</t>
-        </is>
-      </c>
-      <c r="F8" s="3" t="inlineStr">
-        <is>
-          <t>The order-api pod 'order-api-65fdffc6cb-cmmrz' is in CrashLoopBackOff because its 'order-api' container fails to start due to a 'Connection refused' error when trying to connect to 'order-db' (ev_003, ev_004).</t>
-        </is>
-      </c>
-      <c r="G8" t="n">
-        <v>106.1</v>
-      </c>
-      <c r="H8" s="3" t="inlineStr"/>
+      <c r="F8" s="7" t="inlineStr">
+        <is>
+          <t>order-api pods are failing to start because they cannot connect to order-db, receiving a 'Connection refused' error (ev_004).</t>
+        </is>
+      </c>
+      <c r="G8" s="6" t="n">
+        <v>94</v>
+      </c>
+      <c r="H8" s="7" t="inlineStr">
+        <is>
+          <t>Also had no pod name given -- one of the 3 cases that shared the same vulnerability as selector-001. Verified correct both before and after the fix.</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="45" customHeight="1">
       <c r="A9" t="inlineStr">
@@ -905,7 +906,7 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>0.925</v>
+        <v>0.9</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
@@ -919,11 +920,11 @@
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>The pod batch-worker-7 does not exist in the sre-test-cluster, as indicated by multiple 'NotFound' errors (ev_002, ev_004).</t>
+          <t>The pod 'batch-worker-7' does not exist in the 'test-incidents' namespace of 'sre-test-cluster' (ev_002, ev_003).</t>
         </is>
       </c>
       <c r="G9" t="n">
-        <v>88.3</v>
+        <v>35.6</v>
       </c>
       <c r="H9" s="3" t="inlineStr"/>
     </row>
@@ -957,9 +958,13 @@
         </is>
       </c>
       <c r="G10" t="n">
-        <v>8.4</v>
-      </c>
-      <c r="H10" s="3" t="inlineStr"/>
+        <v>7.1</v>
+      </c>
+      <c r="H10" s="3" t="inlineStr">
+        <is>
+          <t>Targets a cluster this agent cannot reach from here, by design. Correctly reports no evidence rather than fabricating a finding.</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="45" customHeight="1">
       <c r="A11" t="inlineStr">
@@ -973,7 +978,7 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>0.825</v>
+        <v>0.65</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
@@ -987,11 +992,11 @@
       </c>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>Pod ghost-pod-42 was deleted, and its associated deployment 'ghost' is also not found, indicating a deletion of the deployment (ev_002, ev_004).</t>
+          <t>The pod 'ghost-pod-42' was not found in the 'sre-test-cluster' (us-central1), indicating it was likely deleted or never existed (ev_001).</t>
         </is>
       </c>
       <c r="G11" t="n">
-        <v>83.7</v>
+        <v>135.9</v>
       </c>
       <c r="H11" s="3" t="inlineStr"/>
     </row>
@@ -1007,25 +1012,25 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>0</v>
+        <v>0.925</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>insufficient_evidence</t>
+          <t>high_confidence</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>insufficient_evidence</t>
+          <t>confirmed</t>
         </is>
       </c>
       <c r="F12" s="3" t="inlineStr">
         <is>
-          <t>The model's response could not be parsed, so no root cause was produced.</t>
+          <t>The pod 'shared-cache-2' does not exist in the 'sre-test-cluster' (us-central1), as confirmed by ev_002.</t>
         </is>
       </c>
       <c r="G12" t="n">
-        <v>120</v>
+        <v>116.6</v>
       </c>
       <c r="H12" s="3" t="inlineStr"/>
     </row>
@@ -1059,9 +1064,13 @@
         </is>
       </c>
       <c r="G13" t="n">
-        <v>4.8</v>
-      </c>
-      <c r="H13" s="3" t="inlineStr"/>
+        <v>12</v>
+      </c>
+      <c r="H13" s="3" t="inlineStr">
+        <is>
+          <t>Deliberately unanswerable query, by design. Correctly and quickly says 'insufficient evidence' rather than guessing -- the right behavior for this case.</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="45" customHeight="1">
       <c r="A14" t="inlineStr">
@@ -1089,11 +1098,11 @@
       </c>
       <c r="F14" s="3" t="inlineStr">
         <is>
-          <t>The pod 'edge-gateway-1' does not exist or was deleted from the 'sre-test-cluster' (ev_001, ev_003).</t>
+          <t>The pod 'edge-gateway-1' does not exist in the 'sre-test-cluster' (us-central1), as confirmed by direct lookup (ev_002).</t>
         </is>
       </c>
       <c r="G14" t="n">
-        <v>45.6</v>
+        <v>38.1</v>
       </c>
       <c r="H14" s="3" t="inlineStr"/>
     </row>
@@ -1109,7 +1118,7 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>0.7</v>
+        <v>0.65</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
@@ -1123,11 +1132,11 @@
       </c>
       <c r="F15" s="3" t="inlineStr">
         <is>
-          <t>The user-service pod failed to start because the 'db-credentials' secret was not found (ev_001, ev_002). This was compounded by initial scheduling failures due to insufficient CPU and untolerated taints (ev_001).</t>
+          <t>The user-service pod is stuck in Pending with CreateContainerConfigError because the 'db-credentials' secret is not found (ev_002, ev_003).</t>
         </is>
       </c>
       <c r="G15" t="n">
-        <v>89.40000000000001</v>
+        <v>90.8</v>
       </c>
       <c r="H15" s="3" t="inlineStr"/>
     </row>

</xml_diff>